<commit_message>
feat: integracion de rol egresado en importacion, gestion y registro publico
- Migracion y base de datos con rol EGRESADO (id 5)
- Soporte en importacion Excel y plantilla descargable con validacion de DNI
- Opcion EGRESADO en creacion/edicion de usuarios en dashboard con badge y filtros
- Formulario publico de autoregistro para egresados en login con diseno de alto contraste
- Endpoint POST /register/graduate con vinculacion de programa de estudio y auto-login
- Permisos para egresados en postulaciones a ofertas, CV y navegacion
</commit_message>
<xml_diff>
--- a/public/assets/Importacion de usuarios.xlsx
+++ b/public/assets/Importacion de usuarios.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="25">
   <si>
     <t>NOMBRES</t>
   </si>
@@ -75,6 +75,21 @@
   </si>
   <si>
     <t>EMPRESA</t>
+  </si>
+  <si>
+    <t>944556677</t>
+  </si>
+  <si>
+    <t>EGRESADO</t>
+  </si>
+  <si>
+    <t>Ana Torres Quispe</t>
+  </si>
+  <si>
+    <t>45678912</t>
+  </si>
+  <si>
+    <t>ana.torres@ejemplo.com</t>
   </si>
 </sst>
 </file>
@@ -562,9 +577,24 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="B6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="7" spans="1:6">
       <c r="B7" s="2"/>
@@ -5542,7 +5572,7 @@
       <formula1>"DNI,RUC,CE"</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Error de rol" error="Por favor seleccione un rol válido: ADMINISTRADOR, DOCENTE, ESTUDIANTE o EMPRESA" promptTitle="Rol" prompt="Seleccione el rol del usuario" sqref="F2:F1000">
-      <formula1>"ADMINISTRADOR,DOCENTE,ESTUDIANTE,EMPRESA"</formula1>
+      <formula1>"ADMINISTRADOR,DOCENTE,ESTUDIANTE,EMPRESA,EGRESADO"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>